<commit_message>
data(auto): atualizacao automatica de impostos e parcelamentos
</commit_message>
<xml_diff>
--- a/parcelamentos_local.xlsx
+++ b/parcelamentos_local.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.121.21.252\controladoria\Vitor\TRIBUTARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{716447C2-D93A-4782-88BA-DF459737AC2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9CD5974-6A16-438D-A85E-745CA3BB4B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="804" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="804" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PARCELAMENTOS" sheetId="1" r:id="rId1"/>
@@ -885,7 +885,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1085,7 +1085,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="3" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2619,10 +2618,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -2661,16 +2660,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$3:$O$3</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$3:$P$3</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>4720740.33</c:v>
                 </c:pt>
@@ -2706,6 +2708,12 @@
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>3912277.58</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5882097.6399999997</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3196894.17</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2742,10 +2750,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -2784,16 +2792,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$4:$O$4</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$4:$P$4</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>749.69</c:v>
                 </c:pt>
@@ -2832,6 +2843,9 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>119.3</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2868,10 +2882,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -2910,16 +2924,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$5:$O$5</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$5:$P$5</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>23389.74</c:v>
                 </c:pt>
@@ -2952,6 +2969,12 @@
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>36214.15</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>53315.91</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>53315.91</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2988,10 +3011,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3030,16 +3053,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$6:$O$6</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$6:$P$6</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>107597.6</c:v>
                 </c:pt>
@@ -3071,13 +3097,16 @@
                   <c:v>111684.99</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>166736.70000000001</c:v>
+                  <c:v>100959.81</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>99037.19</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>245472</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3114,10 +3143,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3156,16 +3185,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$7:$O$7</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$7:$P$7</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>301206.3</c:v>
                 </c:pt>
@@ -3222,10 +3254,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3264,16 +3296,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$8:$O$8</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$8:$P$8</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>99163.88</c:v>
                 </c:pt>
@@ -3350,10 +3385,10 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3392,16 +3427,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$9:$O$9</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$9:$P$9</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>532107.21</c:v>
                 </c:pt>
@@ -3433,13 +3471,16 @@
                   <c:v>136068.29</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>202950.85</c:v>
+                  <c:v>137173.96</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>51.02</c:v>
+                  <c:v>53366.93</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>99156.49</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>298787.91000000003</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4681,15 +4722,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="99" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="102"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="101"/>
     </row>
     <row r="2" spans="1:7" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -4790,22 +4831,22 @@
     </row>
     <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="103" t="s">
+      <c r="A8" s="102" t="s">
         <v>78</v>
       </c>
-      <c r="B8" s="104"/>
-      <c r="C8" s="105"/>
+      <c r="B8" s="103"/>
+      <c r="C8" s="104"/>
       <c r="D8" s="12"/>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="103" t="s">
+      <c r="A9" s="102" t="s">
         <v>97</v>
       </c>
-      <c r="B9" s="104"/>
-      <c r="C9" s="105"/>
+      <c r="B9" s="103"/>
+      <c r="C9" s="104"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
     </row>
@@ -5446,10 +5487,10 @@
         <f>M5-I6</f>
         <v>511198.30999999994</v>
       </c>
-      <c r="O6" s="98" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="98"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.43333314486548447</v>
@@ -5580,11 +5621,11 @@
         <f>M8-I9</f>
         <v>484757.02999999991</v>
       </c>
-      <c r="O9" s="106" t="s">
+      <c r="O9" s="105" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="106"/>
-      <c r="Q9" s="106"/>
+      <c r="P9" s="105"/>
+      <c r="Q9" s="105"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
@@ -5626,11 +5667,11 @@
         <f t="shared" ref="M10:M63" si="2">M9-I10</f>
         <v>475943.2699999999</v>
       </c>
-      <c r="O10" s="107" t="s">
+      <c r="O10" s="106" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="107"/>
-      <c r="Q10" s="107"/>
+      <c r="P10" s="106"/>
+      <c r="Q10" s="106"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
@@ -5672,11 +5713,11 @@
         <f t="shared" si="2"/>
         <v>467129.50999999989</v>
       </c>
-      <c r="O11" s="108" t="s">
+      <c r="O11" s="107" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="108"/>
-      <c r="Q11" s="108"/>
+      <c r="P11" s="107"/>
+      <c r="Q11" s="107"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="83" t="s">
@@ -7482,10 +7523,10 @@
         <f>M5-I6</f>
         <v>1073254.2800000003</v>
       </c>
-      <c r="O6" s="98" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="98"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>Q4/O4-1</f>
         <v>-0.3333332612783364</v>
@@ -7614,11 +7655,11 @@
         <f t="shared" si="2"/>
         <v>1017741.1400000004</v>
       </c>
-      <c r="O9" s="109" t="s">
+      <c r="O9" s="108" t="s">
         <v>86</v>
       </c>
-      <c r="P9" s="109"/>
-      <c r="Q9" s="109"/>
+      <c r="P9" s="108"/>
+      <c r="Q9" s="108"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="79" t="s">
@@ -7660,11 +7701,11 @@
         <f t="shared" si="2"/>
         <v>999236.76000000036</v>
       </c>
-      <c r="O10" s="106" t="s">
+      <c r="O10" s="105" t="s">
         <v>87</v>
       </c>
-      <c r="P10" s="106"/>
-      <c r="Q10" s="106"/>
+      <c r="P10" s="105"/>
+      <c r="Q10" s="105"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="79" t="s">
@@ -7706,11 +7747,11 @@
         <f t="shared" si="2"/>
         <v>980732.38000000035</v>
       </c>
-      <c r="O11" s="107" t="s">
+      <c r="O11" s="106" t="s">
         <v>88</v>
       </c>
-      <c r="P11" s="107"/>
-      <c r="Q11" s="107"/>
+      <c r="P11" s="106"/>
+      <c r="Q11" s="106"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="79" t="s">
@@ -10592,10 +10633,10 @@
         <f>M5-I6</f>
         <v>1727211.77</v>
       </c>
-      <c r="O6" s="98" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="98"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.23333330852134659</v>
@@ -10726,11 +10767,11 @@
         <f t="shared" ref="M9:M63" si="2">M8-I9</f>
         <v>1637873.24</v>
       </c>
-      <c r="O9" s="106" t="s">
+      <c r="O9" s="105" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="106"/>
-      <c r="Q9" s="106"/>
+      <c r="P9" s="105"/>
+      <c r="Q9" s="105"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
@@ -10772,11 +10813,11 @@
         <f t="shared" si="2"/>
         <v>1608093.73</v>
       </c>
-      <c r="O10" s="107" t="s">
+      <c r="O10" s="106" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="107"/>
-      <c r="Q10" s="107"/>
+      <c r="P10" s="106"/>
+      <c r="Q10" s="106"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
@@ -10818,11 +10859,11 @@
         <f t="shared" si="2"/>
         <v>1578314.22</v>
       </c>
-      <c r="O11" s="108" t="s">
+      <c r="O11" s="107" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="108"/>
-      <c r="Q11" s="108"/>
+      <c r="P11" s="107"/>
+      <c r="Q11" s="107"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="81" t="s">
@@ -12594,10 +12635,10 @@
         <f>M5-I6</f>
         <v>88254.450000000012</v>
       </c>
-      <c r="O6" s="98" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="98"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
         <v>-0.14999919494129588</v>
@@ -12683,11 +12724,11 @@
         <f t="shared" ref="M9:M63" si="2">M8-I9</f>
         <v>83689.590000000026</v>
       </c>
-      <c r="O9" s="106" t="s">
+      <c r="O9" s="105" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="106"/>
-      <c r="Q9" s="106"/>
+      <c r="P9" s="105"/>
+      <c r="Q9" s="105"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="39"/>
@@ -12714,11 +12755,11 @@
         <f t="shared" si="2"/>
         <v>82167.97000000003</v>
       </c>
-      <c r="O10" s="107" t="s">
+      <c r="O10" s="106" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="107"/>
-      <c r="Q10" s="107"/>
+      <c r="P10" s="106"/>
+      <c r="Q10" s="106"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="39"/>
@@ -12745,11 +12786,11 @@
         <f t="shared" si="2"/>
         <v>80646.350000000035</v>
       </c>
-      <c r="O11" s="108" t="s">
+      <c r="O11" s="107" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="108"/>
-      <c r="Q11" s="108"/>
+      <c r="P11" s="107"/>
+      <c r="Q11" s="107"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="39"/>
@@ -14348,12 +14389,12 @@
         <v>8285.5799999999963</v>
       </c>
       <c r="P4" s="33">
-        <f>K5+K6</f>
-        <v>516.70000000000005</v>
+        <f>K5+K6+K7+K8+K9+K10+K11+K12+K13+K14+K15</f>
+        <v>2785.48</v>
       </c>
       <c r="Q4" s="34">
         <f>O4-P4</f>
-        <v>7768.8799999999965</v>
+        <v>5500.0999999999967</v>
       </c>
       <c r="R4" s="34">
         <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29</f>
@@ -14411,13 +14452,13 @@
         <f>M5-I6</f>
         <v>-501.4</v>
       </c>
-      <c r="O6" s="98" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="98"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
-        <v>-6.2361355511623806E-2</v>
+        <v>-0.33618406919008692</v>
       </c>
     </row>
     <row r="7" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -14497,9 +14538,9 @@
         <f t="shared" ref="M9:M36" si="1">M8-I9</f>
         <v>-1265.98</v>
       </c>
-      <c r="O9" s="99"/>
-      <c r="P9" s="99"/>
-      <c r="Q9" s="99"/>
+      <c r="O9" s="98"/>
+      <c r="P9" s="98"/>
+      <c r="Q9" s="98"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="39"/>
@@ -14524,9 +14565,9 @@
         <f t="shared" si="1"/>
         <v>-1516.68</v>
       </c>
-      <c r="O10" s="99"/>
-      <c r="P10" s="99"/>
-      <c r="Q10" s="99"/>
+      <c r="O10" s="98"/>
+      <c r="P10" s="98"/>
+      <c r="Q10" s="98"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="39"/>
@@ -14551,9 +14592,9 @@
         <f t="shared" si="1"/>
         <v>-1767.38</v>
       </c>
-      <c r="O11" s="99"/>
-      <c r="P11" s="99"/>
-      <c r="Q11" s="99"/>
+      <c r="O11" s="98"/>
+      <c r="P11" s="98"/>
+      <c r="Q11" s="98"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="39"/>
@@ -15450,30 +15491,30 @@
   <sheetData>
     <row r="1" spans="2:26" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:26" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="111" t="s">
+      <c r="B2" s="110" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="112"/>
-      <c r="D2" s="112"/>
-      <c r="E2" s="112"/>
-      <c r="F2" s="112"/>
-      <c r="G2" s="112"/>
-      <c r="H2" s="112"/>
-      <c r="I2" s="112"/>
-      <c r="J2" s="112"/>
-      <c r="K2" s="112"/>
-      <c r="L2" s="112"/>
-      <c r="M2" s="112"/>
-      <c r="N2" s="112"/>
-      <c r="O2" s="112"/>
-      <c r="P2" s="112"/>
-      <c r="Q2" s="112"/>
-      <c r="R2" s="112"/>
-      <c r="S2" s="112"/>
-      <c r="T2" s="112"/>
-      <c r="U2" s="112"/>
-      <c r="V2" s="112"/>
-      <c r="W2" s="113"/>
+      <c r="C2" s="111"/>
+      <c r="D2" s="111"/>
+      <c r="E2" s="111"/>
+      <c r="F2" s="111"/>
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
+      <c r="J2" s="111"/>
+      <c r="K2" s="111"/>
+      <c r="L2" s="111"/>
+      <c r="M2" s="111"/>
+      <c r="N2" s="111"/>
+      <c r="O2" s="111"/>
+      <c r="P2" s="111"/>
+      <c r="Q2" s="111"/>
+      <c r="R2" s="111"/>
+      <c r="S2" s="111"/>
+      <c r="T2" s="111"/>
+      <c r="U2" s="111"/>
+      <c r="V2" s="111"/>
+      <c r="W2" s="112"/>
     </row>
     <row r="3" spans="2:26" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="48" t="s">
@@ -16304,8 +16345,8 @@
       <c r="Z22" s="57"/>
     </row>
     <row r="24" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P24" s="110"/>
-      <c r="Q24" s="110"/>
+      <c r="P24" s="109"/>
+      <c r="Q24" s="109"/>
       <c r="R24" s="73"/>
       <c r="S24" s="73"/>
       <c r="T24" s="73"/>
@@ -16314,8 +16355,8 @@
       <c r="W24" s="74"/>
     </row>
     <row r="25" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P25" s="110"/>
-      <c r="Q25" s="110"/>
+      <c r="P25" s="109"/>
+      <c r="Q25" s="109"/>
       <c r="R25" s="73"/>
       <c r="S25" s="73"/>
       <c r="T25" s="73"/>
@@ -16324,8 +16365,8 @@
       <c r="W25" s="74"/>
     </row>
     <row r="26" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P26" s="110"/>
-      <c r="Q26" s="110"/>
+      <c r="P26" s="109"/>
+      <c r="Q26" s="109"/>
       <c r="R26" s="73"/>
       <c r="S26" s="73"/>
       <c r="T26" s="73"/>
@@ -16334,8 +16375,8 @@
       <c r="W26" s="74"/>
     </row>
     <row r="27" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P27" s="110"/>
-      <c r="Q27" s="110"/>
+      <c r="P27" s="109"/>
+      <c r="Q27" s="109"/>
       <c r="R27" s="73"/>
       <c r="S27" s="73"/>
       <c r="T27" s="73"/>
@@ -16344,8 +16385,8 @@
       <c r="W27" s="75"/>
     </row>
     <row r="28" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P28" s="110"/>
-      <c r="Q28" s="110"/>
+      <c r="P28" s="109"/>
+      <c r="Q28" s="109"/>
       <c r="R28" s="73"/>
       <c r="S28" s="73"/>
       <c r="T28" s="73"/>
@@ -16371,12 +16412,11 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{420301BD-1EC9-404C-9D58-1869DDAA2327}">
-  <dimension ref="B2:P10"/>
+  <dimension ref="B2:P9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="15" width="13.33203125" customWidth="1"/>
-    <col min="16" max="16" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="16" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.3">
@@ -16419,6 +16459,9 @@
       <c r="O2" s="85">
         <v>46204</v>
       </c>
+      <c r="P2" s="85">
+        <v>46235</v>
+      </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B3" s="84" t="s">
@@ -16464,7 +16507,12 @@
       <c r="N3" s="27">
         <v>3912277.58</v>
       </c>
-      <c r="O3" s="27"/>
+      <c r="O3" s="27">
+        <v>5882097.6399999997</v>
+      </c>
+      <c r="P3" s="27">
+        <v>3196894.17</v>
+      </c>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
@@ -16509,6 +16557,9 @@
       <c r="O4" s="27">
         <v>119.3</v>
       </c>
+      <c r="P4" s="27">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B5" s="84" t="s">
@@ -16549,8 +16600,13 @@
       <c r="M5" s="27">
         <v>36214.15</v>
       </c>
-      <c r="N5" s="27"/>
+      <c r="N5" s="27">
+        <v>53315.91</v>
+      </c>
       <c r="O5" s="27"/>
+      <c r="P5" s="27">
+        <v>53315.91</v>
+      </c>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B6" s="84" t="s">
@@ -16589,13 +16645,16 @@
         <v>111684.99</v>
       </c>
       <c r="M6" s="27">
-        <v>166736.70000000001</v>
+        <v>100959.81</v>
       </c>
       <c r="N6" s="27">
         <v>0</v>
       </c>
       <c r="O6" s="27">
         <v>99037.19</v>
+      </c>
+      <c r="P6" s="27">
+        <v>245472</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.3">
@@ -16631,6 +16690,7 @@
       <c r="M7" s="27"/>
       <c r="N7" s="27"/>
       <c r="O7" s="27"/>
+      <c r="P7" s="27"/>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B8" s="84" t="s">
@@ -16664,6 +16724,7 @@
       <c r="M8" s="27"/>
       <c r="N8" s="27"/>
       <c r="O8" s="27"/>
+      <c r="P8" s="27"/>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B9" s="84" t="s">
@@ -16711,19 +16772,20 @@
       </c>
       <c r="M9" s="96">
         <f t="shared" si="0"/>
-        <v>202950.85</v>
+        <v>137173.96</v>
       </c>
       <c r="N9" s="96">
         <f t="shared" ref="N9:O9" si="1">SUM(N4:N8)</f>
-        <v>51.02</v>
+        <v>53366.93</v>
       </c>
       <c r="O9" s="96">
         <f t="shared" si="1"/>
         <v>99156.49</v>
       </c>
-    </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="P10" s="97"/>
+      <c r="P9" s="96">
+        <f t="shared" ref="P9" si="2">SUM(P4:P8)</f>
+        <v>298787.91000000003</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
data(impostos): atualizacao automatica da base de impostos e parcelamentos
</commit_message>
<xml_diff>
--- a/parcelamentos_local.xlsx
+++ b/parcelamentos_local.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.121.21.252\controladoria\Vitor\TRIBUTARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9CD5974-6A16-438D-A85E-745CA3BB4B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F9FC915-AF91-43AE-8822-E03B7C4443C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="804" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="804" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PARCELAMENTOS" sheetId="1" r:id="rId1"/>
@@ -38,6 +38,69 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={345ACDEE-3A93-4078-BBD5-E741B4EF8544}</author>
+    <author>tc={10D9275D-CEDF-4210-A17E-2431D2A46406}</author>
+    <author>tc={0843B983-A678-4FAC-B87C-05A03C5E6241}</author>
+    <author>tc={DE329B3F-77CB-4B0B-B38B-625328D1F520}</author>
+    <author>tc={F61F0100-07F4-4C2B-8C44-45ED91440663}</author>
+    <author>tc={E3620BFF-2E3F-4954-ABDE-5B5AC2E23EBD}</author>
+  </authors>
+  <commentList>
+    <comment ref="J5" authorId="0" shapeId="0" xr:uid="{345ACDEE-3A93-4078-BBD5-E741B4EF8544}">
+      <text>
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    Feito Perd/Comp com Advogado</t>
+      </text>
+    </comment>
+    <comment ref="K5" authorId="1" shapeId="0" xr:uid="{10D9275D-CEDF-4210-A17E-2431D2A46406}">
+      <text>
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    Feito Perd/Comp com Advogado</t>
+      </text>
+    </comment>
+    <comment ref="L5" authorId="2" shapeId="0" xr:uid="{0843B983-A678-4FAC-B87C-05A03C5E6241}">
+      <text>
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    Feito Perd/Comp com Advogado</t>
+      </text>
+    </comment>
+    <comment ref="J6" authorId="3" shapeId="0" xr:uid="{DE329B3F-77CB-4B0B-B38B-625328D1F520}">
+      <text>
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    Feito Perd/Comp com Advogado</t>
+      </text>
+    </comment>
+    <comment ref="K6" authorId="4" shapeId="0" xr:uid="{F61F0100-07F4-4C2B-8C44-45ED91440663}">
+      <text>
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    Feito Perd/Comp com Advogado</t>
+      </text>
+    </comment>
+    <comment ref="L6" authorId="5" shapeId="0" xr:uid="{E3620BFF-2E3F-4954-ABDE-5B5AC2E23EBD}">
+      <text>
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    Feito Perd/Comp com Advogado</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -364,7 +427,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-&quot;R$&quot;* #,##0.00_-;\-&quot;R$&quot;* #,##0.00_-;_-&quot;R$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -496,6 +559,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="14">
@@ -885,7 +954,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1085,6 +1154,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="3" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2618,10 +2688,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -2660,19 +2730,16 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$3:$P$3</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$3:$O$3</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>4720740.33</c:v>
                 </c:pt>
@@ -2708,12 +2775,6 @@
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>3912277.58</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>5882097.6399999997</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>3196894.17</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2750,10 +2811,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -2792,19 +2853,16 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$4:$P$4</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$4:$O$4</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>749.69</c:v>
                 </c:pt>
@@ -2843,9 +2901,6 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>119.3</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2882,10 +2937,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -2924,19 +2979,16 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$5:$P$5</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$5:$O$5</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>23389.74</c:v>
                 </c:pt>
@@ -2959,22 +3011,16 @@
                   <c:v>22285.39</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>105581.84</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>40560.85</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>24262.02</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>36214.15</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>53315.91</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>53315.91</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3011,10 +3057,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3053,19 +3099,16 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$6:$P$6</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$6:$O$6</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>107597.6</c:v>
                 </c:pt>
@@ -3087,26 +3130,20 @@
                 <c:pt idx="6">
                   <c:v>102854.7</c:v>
                 </c:pt>
-                <c:pt idx="7">
-                  <c:v>486224.38</c:v>
-                </c:pt>
                 <c:pt idx="8">
-                  <c:v>186781.2</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>111684.99</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>100959.81</c:v>
+                  <c:v>166736.70000000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>99037.19</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>245472</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3143,10 +3180,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3185,19 +3222,16 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$7:$P$7</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$7:$O$7</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>301206.3</c:v>
                 </c:pt>
@@ -3254,10 +3288,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3296,19 +3330,16 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$8:$P$8</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$8:$O$8</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>99163.88</c:v>
                 </c:pt>
@@ -3385,10 +3416,10 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3427,19 +3458,16 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$9:$P$9</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$9:$O$9</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="14"/>
+                <c:ptCount val="13"/>
                 <c:pt idx="0">
                   <c:v>532107.21</c:v>
                 </c:pt>
@@ -3462,25 +3490,22 @@
                   <c:v>590640.17999999993</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>591806.22</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>227342.05000000002</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>136068.29</c:v>
+                  <c:v>121.28</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>137173.96</c:v>
+                  <c:v>202950.85</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>53366.93</c:v>
+                  <c:v>51.02</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>99156.49</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>298787.91000000003</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4310,6 +4335,12 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Vitor Cruz" id="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" userId="Vitor Cruz" providerId="None"/>
+</personList>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela3" displayName="Tabela3" ref="A2:G6" totalsRowCount="1" headerRowDxfId="61" dataDxfId="60" totalsRowDxfId="59">
   <autoFilter ref="A2:G5" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
@@ -4699,6 +4730,29 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="J5" dT="2026-09-09T20:56:00.78" personId="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" id="{345ACDEE-3A93-4078-BBD5-E741B4EF8544}">
+    <text>Feito Perd/Comp com Advogado</text>
+  </threadedComment>
+  <threadedComment ref="K5" dT="2026-09-09T20:56:00.78" personId="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" id="{10D9275D-CEDF-4210-A17E-2431D2A46406}">
+    <text>Feito Perd/Comp com Advogado</text>
+  </threadedComment>
+  <threadedComment ref="L5" dT="2026-09-09T20:56:00.78" personId="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" id="{0843B983-A678-4FAC-B87C-05A03C5E6241}">
+    <text>Feito Perd/Comp com Advogado</text>
+  </threadedComment>
+  <threadedComment ref="J6" dT="2026-09-09T20:56:13.78" personId="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" id="{DE329B3F-77CB-4B0B-B38B-625328D1F520}">
+    <text>Feito Perd/Comp com Advogado</text>
+  </threadedComment>
+  <threadedComment ref="K6" dT="2026-09-09T20:56:00.78" personId="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" id="{F61F0100-07F4-4C2B-8C44-45ED91440663}">
+    <text>Feito Perd/Comp com Advogado</text>
+  </threadedComment>
+  <threadedComment ref="L6" dT="2026-09-09T20:56:00.78" personId="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" id="{E3620BFF-2E3F-4954-ABDE-5B5AC2E23EBD}">
+    <text>Feito Perd/Comp com Advogado</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G62"/>
@@ -4722,15 +4776,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="100" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
-      <c r="F1" s="100"/>
-      <c r="G1" s="101"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="101"/>
+      <c r="G1" s="102"/>
     </row>
     <row r="2" spans="1:7" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -4831,22 +4885,22 @@
     </row>
     <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="102" t="s">
+      <c r="A8" s="103" t="s">
         <v>78</v>
       </c>
-      <c r="B8" s="103"/>
-      <c r="C8" s="104"/>
+      <c r="B8" s="104"/>
+      <c r="C8" s="105"/>
       <c r="D8" s="12"/>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="102" t="s">
+      <c r="A9" s="103" t="s">
         <v>97</v>
       </c>
-      <c r="B9" s="103"/>
-      <c r="C9" s="104"/>
+      <c r="B9" s="104"/>
+      <c r="C9" s="105"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
     </row>
@@ -4877,7 +4931,7 @@
       </c>
       <c r="C11" s="17">
         <f>'PARCELAMENTO 06062024'!Q4</f>
-        <v>299668.06999999989</v>
+        <v>290854.30999999988</v>
       </c>
       <c r="D11" s="18" t="s">
         <v>101</v>
@@ -4897,7 +4951,7 @@
       </c>
       <c r="C12" s="17">
         <f>'PARCELAMENTO 05122024'!Q4</f>
-        <v>740175.44</v>
+        <v>721671.06</v>
       </c>
       <c r="D12" s="18" t="s">
         <v>102</v>
@@ -4917,7 +4971,7 @@
       </c>
       <c r="C13" s="17">
         <f>'PARCELAMENTO 06062025'!Q4</f>
-        <v>1369857.65</v>
+        <v>1340078.1399999999</v>
       </c>
       <c r="D13" s="18" t="s">
         <v>98</v>
@@ -4932,7 +4986,7 @@
       <c r="B14" s="20"/>
       <c r="C14" s="89">
         <f>SUM(C11:C13)</f>
-        <v>2409701.1599999997</v>
+        <v>2352603.5099999998</v>
       </c>
       <c r="D14" s="20"/>
       <c r="E14" s="20"/>
@@ -5394,16 +5448,16 @@
         <v>528825.82999999996</v>
       </c>
       <c r="P4" s="33">
-        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18+I19+I20+I21+I22+I23+I24+I25+I26+I27+I28+I29</f>
-        <v>229157.76000000007</v>
+        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18+I19+I20+I21+I22+I23+I24+I25+I26+I27+I28+I29+I30</f>
+        <v>237971.52000000008</v>
       </c>
       <c r="Q4" s="34">
         <f>O4-P4</f>
-        <v>299668.06999999989</v>
+        <v>290854.30999999988</v>
       </c>
       <c r="R4" s="34">
-        <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29</f>
-        <v>28929.75</v>
+        <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29+J30</f>
+        <v>31363.22</v>
       </c>
     </row>
     <row r="5" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -5487,13 +5541,13 @@
         <f>M5-I6</f>
         <v>511198.30999999994</v>
       </c>
-      <c r="O6" s="97" t="s">
+      <c r="O6" s="98" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="97"/>
+      <c r="P6" s="98"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
-        <v>-0.43333314486548447</v>
+        <v>-0.44999980428338782</v>
       </c>
     </row>
     <row r="7" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -5621,11 +5675,11 @@
         <f>M8-I9</f>
         <v>484757.02999999991</v>
       </c>
-      <c r="O9" s="105" t="s">
+      <c r="O9" s="106" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="105"/>
-      <c r="Q9" s="105"/>
+      <c r="P9" s="106"/>
+      <c r="Q9" s="106"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
@@ -5667,11 +5721,11 @@
         <f t="shared" ref="M10:M63" si="2">M9-I10</f>
         <v>475943.2699999999</v>
       </c>
-      <c r="O10" s="106" t="s">
+      <c r="O10" s="107" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="106"/>
-      <c r="Q10" s="106"/>
+      <c r="P10" s="107"/>
+      <c r="Q10" s="107"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
@@ -5713,11 +5767,11 @@
         <f t="shared" si="2"/>
         <v>467129.50999999989</v>
       </c>
-      <c r="O11" s="107" t="s">
+      <c r="O11" s="108" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="107"/>
-      <c r="Q11" s="107"/>
+      <c r="P11" s="108"/>
+      <c r="Q11" s="108"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="83" t="s">
@@ -5869,7 +5923,7 @@
         <v>8813.76</v>
       </c>
       <c r="J15" s="77">
-        <f t="shared" ref="J15:J29" si="3">K15-I15</f>
+        <f t="shared" ref="J15:J30" si="3">K15-I15</f>
         <v>906.93000000000029</v>
       </c>
       <c r="K15" s="28">
@@ -6246,10 +6300,12 @@
       <c r="I30" s="28">
         <v>8813.76</v>
       </c>
-      <c r="J30" s="77"/>
+      <c r="J30" s="77">
+        <f t="shared" si="3"/>
+        <v>2433.4699999999993</v>
+      </c>
       <c r="K30" s="28">
-        <f t="shared" si="1"/>
-        <v>8813.76</v>
+        <v>11247.23</v>
       </c>
       <c r="L30" s="29">
         <v>46265</v>
@@ -7031,11 +7087,11 @@
       </c>
       <c r="J64" s="87">
         <f>SUM(J4:J63)</f>
-        <v>28929.75</v>
+        <v>31363.22</v>
       </c>
       <c r="K64" s="87">
         <f>SUM(K4:K63)</f>
-        <v>557755.58000000019</v>
+        <v>560189.05000000028</v>
       </c>
       <c r="L64" s="43"/>
       <c r="M64" s="44"/>
@@ -7430,16 +7486,16 @@
         <v>1110263.04</v>
       </c>
       <c r="P4" s="33">
-        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18+I19+I20+I21+I22+I23</f>
-        <v>370087.60000000003</v>
+        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18+I19+I20+I21+I22+I23+I24</f>
+        <v>388591.98000000004</v>
       </c>
       <c r="Q4" s="34">
         <f>O4-P4</f>
-        <v>740175.44</v>
+        <v>721671.06</v>
       </c>
       <c r="R4" s="34">
         <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29</f>
-        <v>38411.279999999984</v>
+        <v>42545.14999999998</v>
       </c>
     </row>
     <row r="5" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -7523,13 +7579,13 @@
         <f>M5-I6</f>
         <v>1073254.2800000003</v>
       </c>
-      <c r="O6" s="97" t="s">
+      <c r="O6" s="98" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="97"/>
+      <c r="P6" s="98"/>
       <c r="Q6" s="82">
         <f>Q4/O4-1</f>
-        <v>-0.3333332612783364</v>
+        <v>-0.34999992434225313</v>
       </c>
     </row>
     <row r="7" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -7642,7 +7698,7 @@
         <v>18504.38</v>
       </c>
       <c r="J9" s="28">
-        <f t="shared" ref="J9:J23" si="3">K9-I9</f>
+        <f t="shared" ref="J9:J24" si="3">K9-I9</f>
         <v>928.90999999999985</v>
       </c>
       <c r="K9" s="28">
@@ -7655,11 +7711,11 @@
         <f t="shared" si="2"/>
         <v>1017741.1400000004</v>
       </c>
-      <c r="O9" s="108" t="s">
+      <c r="O9" s="109" t="s">
         <v>86</v>
       </c>
-      <c r="P9" s="108"/>
-      <c r="Q9" s="108"/>
+      <c r="P9" s="109"/>
+      <c r="Q9" s="109"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="79" t="s">
@@ -7701,11 +7757,11 @@
         <f t="shared" si="2"/>
         <v>999236.76000000036</v>
       </c>
-      <c r="O10" s="105" t="s">
+      <c r="O10" s="106" t="s">
         <v>87</v>
       </c>
-      <c r="P10" s="105"/>
-      <c r="Q10" s="105"/>
+      <c r="P10" s="106"/>
+      <c r="Q10" s="106"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="79" t="s">
@@ -7747,11 +7803,11 @@
         <f t="shared" si="2"/>
         <v>980732.38000000035</v>
       </c>
-      <c r="O11" s="106" t="s">
+      <c r="O11" s="107" t="s">
         <v>88</v>
       </c>
-      <c r="P11" s="106"/>
-      <c r="Q11" s="106"/>
+      <c r="P11" s="107"/>
+      <c r="Q11" s="107"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="79" t="s">
@@ -8282,8 +8338,13 @@
       <c r="I24" s="28">
         <v>18504.38</v>
       </c>
-      <c r="J24" s="28"/>
-      <c r="K24" s="28"/>
+      <c r="J24" s="28">
+        <f t="shared" si="3"/>
+        <v>4133.869999999999</v>
+      </c>
+      <c r="K24" s="28">
+        <v>22638.25</v>
+      </c>
       <c r="L24" s="29">
         <v>46265</v>
       </c>
@@ -9616,11 +9677,11 @@
       </c>
       <c r="J64" s="78">
         <f>SUM(J4:J63)</f>
-        <v>38411.279999999984</v>
+        <v>42545.14999999998</v>
       </c>
       <c r="K64" s="78">
         <f>SUM(K4:K63)</f>
-        <v>389994.5</v>
+        <v>412632.75</v>
       </c>
       <c r="L64" s="43"/>
       <c r="M64" s="44"/>
@@ -10540,16 +10601,16 @@
         <v>1786770.79</v>
       </c>
       <c r="P4" s="33">
-        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17</f>
-        <v>416913.14000000007</v>
+        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18</f>
+        <v>446692.65000000008</v>
       </c>
       <c r="Q4" s="34">
         <f>O4-P4</f>
-        <v>1369857.65</v>
+        <v>1340078.1399999999</v>
       </c>
       <c r="R4" s="34">
         <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29</f>
-        <v>31664.490000000016</v>
+        <v>36453.030000000021</v>
       </c>
     </row>
     <row r="5" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -10579,7 +10640,7 @@
         <v>29779.51</v>
       </c>
       <c r="J5" s="77">
-        <f t="shared" ref="J5:J17" si="1">K5-I5</f>
+        <f t="shared" ref="J5:J18" si="1">K5-I5</f>
         <v>297.79000000000087</v>
       </c>
       <c r="K5" s="28">
@@ -10633,13 +10694,13 @@
         <f>M5-I6</f>
         <v>1727211.77</v>
       </c>
-      <c r="O6" s="97" t="s">
+      <c r="O6" s="98" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="97"/>
+      <c r="P6" s="98"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
-        <v>-0.23333330852134659</v>
+        <v>-0.24999997341572844</v>
       </c>
     </row>
     <row r="7" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -10767,11 +10828,11 @@
         <f t="shared" ref="M9:M63" si="2">M8-I9</f>
         <v>1637873.24</v>
       </c>
-      <c r="O9" s="105" t="s">
+      <c r="O9" s="106" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="105"/>
-      <c r="Q9" s="105"/>
+      <c r="P9" s="106"/>
+      <c r="Q9" s="106"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
@@ -10813,11 +10874,11 @@
         <f t="shared" si="2"/>
         <v>1608093.73</v>
       </c>
-      <c r="O10" s="106" t="s">
+      <c r="O10" s="107" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="106"/>
-      <c r="Q10" s="106"/>
+      <c r="P10" s="107"/>
+      <c r="Q10" s="107"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
@@ -10859,11 +10920,11 @@
         <f t="shared" si="2"/>
         <v>1578314.22</v>
       </c>
-      <c r="O11" s="107" t="s">
+      <c r="O11" s="108" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="107"/>
-      <c r="Q11" s="107"/>
+      <c r="P11" s="108"/>
+      <c r="Q11" s="108"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="81" t="s">
@@ -11108,10 +11169,12 @@
       <c r="I18" s="28">
         <v>29779.51</v>
       </c>
-      <c r="J18" s="77"/>
+      <c r="J18" s="77">
+        <f t="shared" si="1"/>
+        <v>4788.5400000000045</v>
+      </c>
       <c r="K18" s="28">
-        <f t="shared" ref="K18:K63" si="3">I18+J18</f>
-        <v>29779.51</v>
+        <v>34568.050000000003</v>
       </c>
       <c r="L18" s="29">
         <v>45900</v>
@@ -11133,7 +11196,7 @@
       </c>
       <c r="J19" s="77"/>
       <c r="K19" s="28">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="K19:K63" si="3">I19+J19</f>
         <v>29779.51</v>
       </c>
       <c r="L19" s="29">
@@ -12169,11 +12232,11 @@
       </c>
       <c r="J64" s="78">
         <f>SUM(J4:J63)</f>
-        <v>31664.490000000016</v>
+        <v>36453.030000000021</v>
       </c>
       <c r="K64" s="78">
         <f>SUM(K4:K63)</f>
-        <v>1818435.2800000003</v>
+        <v>1823223.8200000003</v>
       </c>
       <c r="L64" s="43"/>
       <c r="M64" s="44"/>
@@ -12571,16 +12634,16 @@
         <v>91297.69</v>
       </c>
       <c r="P4" s="33">
-        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12</f>
-        <v>13694.579999999998</v>
+        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13</f>
+        <v>15216.199999999997</v>
       </c>
       <c r="Q4" s="34">
         <f>O4-P4</f>
-        <v>77603.11</v>
+        <v>76081.490000000005</v>
       </c>
       <c r="R4" s="34">
         <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29</f>
-        <v>591.41000000000076</v>
+        <v>744.94000000000096</v>
       </c>
     </row>
     <row r="5" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -12622,7 +12685,7 @@
         <v>1521.62</v>
       </c>
       <c r="J6" s="77">
-        <f t="shared" ref="J6:J12" si="1">K6-I6</f>
+        <f t="shared" ref="J6:J13" si="1">K6-I6</f>
         <v>33.770000000000209</v>
       </c>
       <c r="K6" s="28">
@@ -12635,13 +12698,13 @@
         <f>M5-I6</f>
         <v>88254.450000000012</v>
       </c>
-      <c r="O6" s="97" t="s">
+      <c r="O6" s="98" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="97"/>
+      <c r="P6" s="98"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
-        <v>-0.14999919494129588</v>
+        <v>-0.16666577215699541</v>
       </c>
     </row>
     <row r="7" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -12724,11 +12787,11 @@
         <f t="shared" ref="M9:M63" si="2">M8-I9</f>
         <v>83689.590000000026</v>
       </c>
-      <c r="O9" s="105" t="s">
+      <c r="O9" s="106" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="105"/>
-      <c r="Q9" s="105"/>
+      <c r="P9" s="106"/>
+      <c r="Q9" s="106"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="39"/>
@@ -12755,11 +12818,11 @@
         <f t="shared" si="2"/>
         <v>82167.97000000003</v>
       </c>
-      <c r="O10" s="106" t="s">
+      <c r="O10" s="107" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="106"/>
-      <c r="Q10" s="106"/>
+      <c r="P10" s="107"/>
+      <c r="Q10" s="107"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="39"/>
@@ -12786,11 +12849,11 @@
         <f t="shared" si="2"/>
         <v>80646.350000000035</v>
       </c>
-      <c r="O11" s="107" t="s">
+      <c r="O11" s="108" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="107"/>
-      <c r="Q11" s="107"/>
+      <c r="P11" s="108"/>
+      <c r="Q11" s="108"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="39"/>
@@ -12829,10 +12892,12 @@
       <c r="I13" s="27">
         <v>1521.62</v>
       </c>
-      <c r="J13" s="77"/>
+      <c r="J13" s="77">
+        <f t="shared" si="1"/>
+        <v>153.5300000000002</v>
+      </c>
       <c r="K13" s="28">
-        <f t="shared" si="0"/>
-        <v>1521.62</v>
+        <v>1675.15</v>
       </c>
       <c r="L13" s="29">
         <v>46262</v>
@@ -14389,12 +14454,12 @@
         <v>8285.5799999999963</v>
       </c>
       <c r="P4" s="33">
-        <f>K5+K6+K7+K8+K9+K10+K11+K12+K13+K14+K15</f>
-        <v>2785.48</v>
+        <f>K5+K6</f>
+        <v>516.70000000000005</v>
       </c>
       <c r="Q4" s="34">
         <f>O4-P4</f>
-        <v>5500.0999999999967</v>
+        <v>7768.8799999999965</v>
       </c>
       <c r="R4" s="34">
         <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29</f>
@@ -14452,13 +14517,13 @@
         <f>M5-I6</f>
         <v>-501.4</v>
       </c>
-      <c r="O6" s="97" t="s">
+      <c r="O6" s="98" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="97"/>
+      <c r="P6" s="98"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
-        <v>-0.33618406919008692</v>
+        <v>-6.2361355511623806E-2</v>
       </c>
     </row>
     <row r="7" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -14538,9 +14603,9 @@
         <f t="shared" ref="M9:M36" si="1">M8-I9</f>
         <v>-1265.98</v>
       </c>
-      <c r="O9" s="98"/>
-      <c r="P9" s="98"/>
-      <c r="Q9" s="98"/>
+      <c r="O9" s="99"/>
+      <c r="P9" s="99"/>
+      <c r="Q9" s="99"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="39"/>
@@ -14565,9 +14630,9 @@
         <f t="shared" si="1"/>
         <v>-1516.68</v>
       </c>
-      <c r="O10" s="98"/>
-      <c r="P10" s="98"/>
-      <c r="Q10" s="98"/>
+      <c r="O10" s="99"/>
+      <c r="P10" s="99"/>
+      <c r="Q10" s="99"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="39"/>
@@ -14592,9 +14657,9 @@
         <f t="shared" si="1"/>
         <v>-1767.38</v>
       </c>
-      <c r="O11" s="98"/>
-      <c r="P11" s="98"/>
-      <c r="Q11" s="98"/>
+      <c r="O11" s="99"/>
+      <c r="P11" s="99"/>
+      <c r="Q11" s="99"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="39"/>
@@ -15491,30 +15556,30 @@
   <sheetData>
     <row r="1" spans="2:26" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:26" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="110" t="s">
+      <c r="B2" s="111" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="111"/>
-      <c r="D2" s="111"/>
-      <c r="E2" s="111"/>
-      <c r="F2" s="111"/>
-      <c r="G2" s="111"/>
-      <c r="H2" s="111"/>
-      <c r="I2" s="111"/>
-      <c r="J2" s="111"/>
-      <c r="K2" s="111"/>
-      <c r="L2" s="111"/>
-      <c r="M2" s="111"/>
-      <c r="N2" s="111"/>
-      <c r="O2" s="111"/>
-      <c r="P2" s="111"/>
-      <c r="Q2" s="111"/>
-      <c r="R2" s="111"/>
-      <c r="S2" s="111"/>
-      <c r="T2" s="111"/>
-      <c r="U2" s="111"/>
-      <c r="V2" s="111"/>
-      <c r="W2" s="112"/>
+      <c r="C2" s="112"/>
+      <c r="D2" s="112"/>
+      <c r="E2" s="112"/>
+      <c r="F2" s="112"/>
+      <c r="G2" s="112"/>
+      <c r="H2" s="112"/>
+      <c r="I2" s="112"/>
+      <c r="J2" s="112"/>
+      <c r="K2" s="112"/>
+      <c r="L2" s="112"/>
+      <c r="M2" s="112"/>
+      <c r="N2" s="112"/>
+      <c r="O2" s="112"/>
+      <c r="P2" s="112"/>
+      <c r="Q2" s="112"/>
+      <c r="R2" s="112"/>
+      <c r="S2" s="112"/>
+      <c r="T2" s="112"/>
+      <c r="U2" s="112"/>
+      <c r="V2" s="112"/>
+      <c r="W2" s="113"/>
     </row>
     <row r="3" spans="2:26" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="48" t="s">
@@ -16345,8 +16410,8 @@
       <c r="Z22" s="57"/>
     </row>
     <row r="24" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P24" s="109"/>
-      <c r="Q24" s="109"/>
+      <c r="P24" s="110"/>
+      <c r="Q24" s="110"/>
       <c r="R24" s="73"/>
       <c r="S24" s="73"/>
       <c r="T24" s="73"/>
@@ -16355,8 +16420,8 @@
       <c r="W24" s="74"/>
     </row>
     <row r="25" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P25" s="109"/>
-      <c r="Q25" s="109"/>
+      <c r="P25" s="110"/>
+      <c r="Q25" s="110"/>
       <c r="R25" s="73"/>
       <c r="S25" s="73"/>
       <c r="T25" s="73"/>
@@ -16365,8 +16430,8 @@
       <c r="W25" s="74"/>
     </row>
     <row r="26" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P26" s="109"/>
-      <c r="Q26" s="109"/>
+      <c r="P26" s="110"/>
+      <c r="Q26" s="110"/>
       <c r="R26" s="73"/>
       <c r="S26" s="73"/>
       <c r="T26" s="73"/>
@@ -16375,8 +16440,8 @@
       <c r="W26" s="74"/>
     </row>
     <row r="27" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P27" s="109"/>
-      <c r="Q27" s="109"/>
+      <c r="P27" s="110"/>
+      <c r="Q27" s="110"/>
       <c r="R27" s="73"/>
       <c r="S27" s="73"/>
       <c r="T27" s="73"/>
@@ -16385,8 +16450,8 @@
       <c r="W27" s="75"/>
     </row>
     <row r="28" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P28" s="109"/>
-      <c r="Q28" s="109"/>
+      <c r="P28" s="110"/>
+      <c r="Q28" s="110"/>
       <c r="R28" s="73"/>
       <c r="S28" s="73"/>
       <c r="T28" s="73"/>
@@ -16411,12 +16476,13 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{420301BD-1EC9-404C-9D58-1869DDAA2327}">
-  <dimension ref="B2:P9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{420301BD-1EC9-404C-9D58-1869DDAA2327}">
+  <dimension ref="B2:P10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="16" width="13.33203125" customWidth="1"/>
+    <col min="3" max="15" width="13.33203125" customWidth="1"/>
+    <col min="16" max="16" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.3">
@@ -16459,9 +16525,6 @@
       <c r="O2" s="85">
         <v>46204</v>
       </c>
-      <c r="P2" s="85">
-        <v>46235</v>
-      </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B3" s="84" t="s">
@@ -16507,12 +16570,7 @@
       <c r="N3" s="27">
         <v>3912277.58</v>
       </c>
-      <c r="O3" s="27">
-        <v>5882097.6399999997</v>
-      </c>
-      <c r="P3" s="27">
-        <v>3196894.17</v>
-      </c>
+      <c r="O3" s="27"/>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
@@ -16557,9 +16615,6 @@
       <c r="O4" s="27">
         <v>119.3</v>
       </c>
-      <c r="P4" s="27">
-        <v>0</v>
-      </c>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B5" s="84" t="s">
@@ -16588,25 +16643,19 @@
         <v>22285.39</v>
       </c>
       <c r="J5" s="27">
-        <v>105581.84</v>
+        <v>0</v>
       </c>
       <c r="K5" s="27">
-        <v>40560.85</v>
+        <v>0</v>
       </c>
       <c r="L5" s="27">
-        <f>24262.02</f>
-        <v>24262.02</v>
+        <v>0</v>
       </c>
       <c r="M5" s="27">
         <v>36214.15</v>
       </c>
-      <c r="N5" s="27">
-        <v>53315.91</v>
-      </c>
+      <c r="N5" s="27"/>
       <c r="O5" s="27"/>
-      <c r="P5" s="27">
-        <v>53315.91</v>
-      </c>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B6" s="84" t="s">
@@ -16634,27 +16683,21 @@
         <f>102854.7</f>
         <v>102854.7</v>
       </c>
-      <c r="J6" s="27">
-        <v>486224.38</v>
-      </c>
+      <c r="J6" s="27"/>
       <c r="K6" s="27">
-        <v>186781.2</v>
+        <v>0</v>
       </c>
       <c r="L6" s="27">
-        <f>111684.99</f>
-        <v>111684.99</v>
+        <v>0</v>
       </c>
       <c r="M6" s="27">
-        <v>100959.81</v>
+        <v>166736.70000000001</v>
       </c>
       <c r="N6" s="27">
         <v>0</v>
       </c>
       <c r="O6" s="27">
         <v>99037.19</v>
-      </c>
-      <c r="P6" s="27">
-        <v>245472</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.3">
@@ -16690,7 +16733,6 @@
       <c r="M7" s="27"/>
       <c r="N7" s="27"/>
       <c r="O7" s="27"/>
-      <c r="P7" s="27"/>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B8" s="84" t="s">
@@ -16724,7 +16766,6 @@
       <c r="M8" s="27"/>
       <c r="N8" s="27"/>
       <c r="O8" s="27"/>
-      <c r="P8" s="27"/>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B9" s="84" t="s">
@@ -16760,35 +16801,35 @@
       </c>
       <c r="J9" s="96">
         <f t="shared" si="0"/>
-        <v>591806.22</v>
+        <v>0</v>
       </c>
       <c r="K9" s="96">
         <f t="shared" si="0"/>
-        <v>227342.05000000002</v>
+        <v>0</v>
       </c>
       <c r="L9" s="96">
         <f t="shared" si="0"/>
-        <v>136068.29</v>
+        <v>121.28</v>
       </c>
       <c r="M9" s="96">
         <f t="shared" si="0"/>
-        <v>137173.96</v>
+        <v>202950.85</v>
       </c>
       <c r="N9" s="96">
         <f t="shared" ref="N9:O9" si="1">SUM(N4:N8)</f>
-        <v>53366.93</v>
+        <v>51.02</v>
       </c>
       <c r="O9" s="96">
         <f t="shared" si="1"/>
         <v>99156.49</v>
       </c>
-      <c r="P9" s="96">
-        <f t="shared" ref="P9" si="2">SUM(P4:P8)</f>
-        <v>298787.91000000003</v>
-      </c>
+    </row>
+    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
+      <c r="P10" s="97"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(impostos): ajuste da apuracao tributaria e parcelamentos conforme planilha atualizada
</commit_message>
<xml_diff>
--- a/parcelamentos_local.xlsx
+++ b/parcelamentos_local.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\10.121.21.252\controladoria\Vitor\TRIBUTARIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F9FC915-AF91-43AE-8822-E03B7C4443C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B201C1-5488-4682-B60D-E2E40722776C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="804" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,15 +43,15 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={345ACDEE-3A93-4078-BBD5-E741B4EF8544}</author>
-    <author>tc={10D9275D-CEDF-4210-A17E-2431D2A46406}</author>
-    <author>tc={0843B983-A678-4FAC-B87C-05A03C5E6241}</author>
-    <author>tc={DE329B3F-77CB-4B0B-B38B-625328D1F520}</author>
-    <author>tc={F61F0100-07F4-4C2B-8C44-45ED91440663}</author>
-    <author>tc={E3620BFF-2E3F-4954-ABDE-5B5AC2E23EBD}</author>
+    <author>tc={79A807FC-C033-4AD6-B2F3-3D2118AA2844}</author>
+    <author>tc={2820BD41-D688-4477-BDC3-A2CC3F279BE1}</author>
+    <author>tc={69B0B8BE-7EBE-4A56-BED3-52263843B1C3}</author>
+    <author>tc={704F14D4-648A-4488-8D55-88B91691F4FE}</author>
+    <author>tc={4C44609A-B8C3-4280-ABA6-12D52E40642B}</author>
+    <author>tc={EA2F0DAC-E08D-4AB3-95AC-6E387F78470E}</author>
   </authors>
   <commentList>
-    <comment ref="J5" authorId="0" shapeId="0" xr:uid="{345ACDEE-3A93-4078-BBD5-E741B4EF8544}">
+    <comment ref="J5" authorId="0" shapeId="0" xr:uid="{79A807FC-C033-4AD6-B2F3-3D2118AA2844}">
       <text>
         <t>[Comentário encadeado]
 Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
@@ -59,7 +59,7 @@
     Feito Perd/Comp com Advogado</t>
       </text>
     </comment>
-    <comment ref="K5" authorId="1" shapeId="0" xr:uid="{10D9275D-CEDF-4210-A17E-2431D2A46406}">
+    <comment ref="K5" authorId="1" shapeId="0" xr:uid="{2820BD41-D688-4477-BDC3-A2CC3F279BE1}">
       <text>
         <t>[Comentário encadeado]
 Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
@@ -67,7 +67,7 @@
     Feito Perd/Comp com Advogado</t>
       </text>
     </comment>
-    <comment ref="L5" authorId="2" shapeId="0" xr:uid="{0843B983-A678-4FAC-B87C-05A03C5E6241}">
+    <comment ref="L5" authorId="2" shapeId="0" xr:uid="{69B0B8BE-7EBE-4A56-BED3-52263843B1C3}">
       <text>
         <t>[Comentário encadeado]
 Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
@@ -75,7 +75,7 @@
     Feito Perd/Comp com Advogado</t>
       </text>
     </comment>
-    <comment ref="J6" authorId="3" shapeId="0" xr:uid="{DE329B3F-77CB-4B0B-B38B-625328D1F520}">
+    <comment ref="J6" authorId="3" shapeId="0" xr:uid="{704F14D4-648A-4488-8D55-88B91691F4FE}">
       <text>
         <t>[Comentário encadeado]
 Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
@@ -83,7 +83,7 @@
     Feito Perd/Comp com Advogado</t>
       </text>
     </comment>
-    <comment ref="K6" authorId="4" shapeId="0" xr:uid="{F61F0100-07F4-4C2B-8C44-45ED91440663}">
+    <comment ref="K6" authorId="4" shapeId="0" xr:uid="{4C44609A-B8C3-4280-ABA6-12D52E40642B}">
       <text>
         <t>[Comentário encadeado]
 Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
@@ -91,7 +91,7 @@
     Feito Perd/Comp com Advogado</t>
       </text>
     </comment>
-    <comment ref="L6" authorId="5" shapeId="0" xr:uid="{E3620BFF-2E3F-4954-ABDE-5B5AC2E23EBD}">
+    <comment ref="L6" authorId="5" shapeId="0" xr:uid="{EA2F0DAC-E08D-4AB3-95AC-6E387F78470E}">
       <text>
         <t>[Comentário encadeado]
 Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
@@ -422,10 +422,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-&quot;R$&quot;* #,##0.00_-;\-&quot;R$&quot;* #,##0.00_-;_-&quot;R$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -948,13 +950,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1154,7 +1158,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="3" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1204,11 +1207,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="6">
     <cellStyle name="Moeda" xfId="2" builtinId="4"/>
+    <cellStyle name="Moeda 2" xfId="5" xr:uid="{239B096F-C6C3-43AA-9629-E08B06BF09A1}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="3" builtinId="5"/>
     <cellStyle name="Vírgula" xfId="1" builtinId="3"/>
+    <cellStyle name="Vírgula 2" xfId="4" xr:uid="{44236E6F-F78E-409C-B867-8BADB28E2B91}"/>
   </cellStyles>
   <dxfs count="62">
     <dxf>
@@ -2688,10 +2693,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -2730,16 +2735,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$3:$O$3</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$3:$P$3</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>4720740.33</c:v>
                 </c:pt>
@@ -2775,6 +2783,12 @@
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>3912277.58</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5882097.6399999997</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3196894.17</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2811,10 +2825,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -2853,16 +2867,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$4:$O$4</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$4:$P$4</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>749.69</c:v>
                 </c:pt>
@@ -2901,6 +2918,9 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>119.3</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2937,10 +2957,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -2979,16 +2999,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$5:$O$5</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$5:$P$5</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>23389.74</c:v>
                 </c:pt>
@@ -3021,6 +3044,12 @@
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>36214.15</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>53315.91</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>53315.91</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3057,10 +3086,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3099,16 +3128,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$6:$O$6</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$6:$P$6</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>107597.6</c:v>
                 </c:pt>
@@ -3130,6 +3162,9 @@
                 <c:pt idx="6">
                   <c:v>102854.7</c:v>
                 </c:pt>
+                <c:pt idx="7">
+                  <c:v>0</c:v>
+                </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
                 </c:pt>
@@ -3137,13 +3172,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>166736.70000000001</c:v>
+                  <c:v>100959.81</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>99037.19</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>245472</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3180,10 +3218,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3222,16 +3260,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$7:$O$7</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$7:$P$7</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>301206.3</c:v>
                 </c:pt>
@@ -3288,10 +3329,10 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3330,16 +3371,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$8:$O$8</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$8:$P$8</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>99163.88</c:v>
                 </c:pt>
@@ -3416,10 +3460,10 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$O$2</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$2:$P$2</c:f>
               <c:numCache>
                 <c:formatCode>mmm\-yy</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>45839</c:v>
                 </c:pt>
@@ -3458,16 +3502,19 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>46204</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46235</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'ACOMPANHAMENTO MENSAL'!$C$9:$O$9</c:f>
+              <c:f>'ACOMPANHAMENTO MENSAL'!$C$9:$P$9</c:f>
               <c:numCache>
                 <c:formatCode>_(* #,##0.00_);_(* \(#,##0.00\);_(* "-"??_);_(@_)</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>532107.21</c:v>
                 </c:pt>
@@ -3499,13 +3546,16 @@
                   <c:v>121.28</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>202950.85</c:v>
+                  <c:v>137173.96</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>51.02</c:v>
+                  <c:v>53366.93</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>99156.49</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>298787.91000000003</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4337,7 +4387,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Vitor Cruz" id="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" userId="Vitor Cruz" providerId="None"/>
+  <person displayName="Vitor Cruz" id="{595D0C01-13C6-47BC-9C7D-36DE33B86AC0}" userId="Vitor Cruz" providerId="None"/>
 </personList>
 </file>
 
@@ -4732,22 +4782,22 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="J5" dT="2026-09-09T20:56:00.78" personId="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" id="{345ACDEE-3A93-4078-BBD5-E741B4EF8544}">
+  <threadedComment ref="J5" dT="2026-09-09T20:56:00.78" personId="{595D0C01-13C6-47BC-9C7D-36DE33B86AC0}" id="{79A807FC-C033-4AD6-B2F3-3D2118AA2844}">
     <text>Feito Perd/Comp com Advogado</text>
   </threadedComment>
-  <threadedComment ref="K5" dT="2026-09-09T20:56:00.78" personId="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" id="{10D9275D-CEDF-4210-A17E-2431D2A46406}">
+  <threadedComment ref="K5" dT="2026-09-09T20:56:00.78" personId="{595D0C01-13C6-47BC-9C7D-36DE33B86AC0}" id="{2820BD41-D688-4477-BDC3-A2CC3F279BE1}">
     <text>Feito Perd/Comp com Advogado</text>
   </threadedComment>
-  <threadedComment ref="L5" dT="2026-09-09T20:56:00.78" personId="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" id="{0843B983-A678-4FAC-B87C-05A03C5E6241}">
+  <threadedComment ref="L5" dT="2026-09-09T20:56:00.78" personId="{595D0C01-13C6-47BC-9C7D-36DE33B86AC0}" id="{69B0B8BE-7EBE-4A56-BED3-52263843B1C3}">
     <text>Feito Perd/Comp com Advogado</text>
   </threadedComment>
-  <threadedComment ref="J6" dT="2026-09-09T20:56:13.78" personId="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" id="{DE329B3F-77CB-4B0B-B38B-625328D1F520}">
+  <threadedComment ref="J6" dT="2026-09-09T20:56:00.78" personId="{595D0C01-13C6-47BC-9C7D-36DE33B86AC0}" id="{704F14D4-648A-4488-8D55-88B91691F4FE}">
     <text>Feito Perd/Comp com Advogado</text>
   </threadedComment>
-  <threadedComment ref="K6" dT="2026-09-09T20:56:00.78" personId="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" id="{F61F0100-07F4-4C2B-8C44-45ED91440663}">
+  <threadedComment ref="K6" dT="2026-09-09T20:56:00.78" personId="{595D0C01-13C6-47BC-9C7D-36DE33B86AC0}" id="{4C44609A-B8C3-4280-ABA6-12D52E40642B}">
     <text>Feito Perd/Comp com Advogado</text>
   </threadedComment>
-  <threadedComment ref="L6" dT="2026-09-09T20:56:00.78" personId="{5860D5EA-0478-41C9-BF5A-4C074234F96B}" id="{E3620BFF-2E3F-4954-ABDE-5B5AC2E23EBD}">
+  <threadedComment ref="L6" dT="2026-09-09T20:56:00.78" personId="{595D0C01-13C6-47BC-9C7D-36DE33B86AC0}" id="{EA2F0DAC-E08D-4AB3-95AC-6E387F78470E}">
     <text>Feito Perd/Comp com Advogado</text>
   </threadedComment>
 </ThreadedComments>
@@ -4776,15 +4826,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.75" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="99" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="101"/>
-      <c r="E1" s="101"/>
-      <c r="F1" s="101"/>
-      <c r="G1" s="102"/>
+      <c r="B1" s="100"/>
+      <c r="C1" s="100"/>
+      <c r="D1" s="100"/>
+      <c r="E1" s="100"/>
+      <c r="F1" s="100"/>
+      <c r="G1" s="101"/>
     </row>
     <row r="2" spans="1:7" s="4" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -4885,22 +4935,22 @@
     </row>
     <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="8" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="103" t="s">
+      <c r="A8" s="102" t="s">
         <v>78</v>
       </c>
-      <c r="B8" s="104"/>
-      <c r="C8" s="105"/>
+      <c r="B8" s="103"/>
+      <c r="C8" s="104"/>
       <c r="D8" s="12"/>
       <c r="E8" s="12"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
     </row>
     <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="103" t="s">
+      <c r="A9" s="102" t="s">
         <v>97</v>
       </c>
-      <c r="B9" s="104"/>
-      <c r="C9" s="105"/>
+      <c r="B9" s="103"/>
+      <c r="C9" s="104"/>
       <c r="D9" s="13"/>
       <c r="E9" s="13"/>
     </row>
@@ -4931,7 +4981,7 @@
       </c>
       <c r="C11" s="17">
         <f>'PARCELAMENTO 06062024'!Q4</f>
-        <v>290854.30999999988</v>
+        <v>299668.06999999989</v>
       </c>
       <c r="D11" s="18" t="s">
         <v>101</v>
@@ -4951,7 +5001,7 @@
       </c>
       <c r="C12" s="17">
         <f>'PARCELAMENTO 05122024'!Q4</f>
-        <v>721671.06</v>
+        <v>740175.44</v>
       </c>
       <c r="D12" s="18" t="s">
         <v>102</v>
@@ -4971,7 +5021,7 @@
       </c>
       <c r="C13" s="17">
         <f>'PARCELAMENTO 06062025'!Q4</f>
-        <v>1340078.1399999999</v>
+        <v>1369857.65</v>
       </c>
       <c r="D13" s="18" t="s">
         <v>98</v>
@@ -4986,7 +5036,7 @@
       <c r="B14" s="20"/>
       <c r="C14" s="89">
         <f>SUM(C11:C13)</f>
-        <v>2352603.5099999998</v>
+        <v>2409701.1599999997</v>
       </c>
       <c r="D14" s="20"/>
       <c r="E14" s="20"/>
@@ -5448,16 +5498,16 @@
         <v>528825.82999999996</v>
       </c>
       <c r="P4" s="33">
-        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18+I19+I20+I21+I22+I23+I24+I25+I26+I27+I28+I29+I30</f>
-        <v>237971.52000000008</v>
+        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18+I19+I20+I21+I22+I23+I24+I25+I26+I27+I28+I29</f>
+        <v>229157.76000000007</v>
       </c>
       <c r="Q4" s="34">
         <f>O4-P4</f>
-        <v>290854.30999999988</v>
+        <v>299668.06999999989</v>
       </c>
       <c r="R4" s="34">
-        <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29+J30</f>
-        <v>31363.22</v>
+        <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29</f>
+        <v>28929.75</v>
       </c>
     </row>
     <row r="5" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -5541,13 +5591,13 @@
         <f>M5-I6</f>
         <v>511198.30999999994</v>
       </c>
-      <c r="O6" s="98" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="98"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
-        <v>-0.44999980428338782</v>
+        <v>-0.43333314486548447</v>
       </c>
     </row>
     <row r="7" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -5675,11 +5725,11 @@
         <f>M8-I9</f>
         <v>484757.02999999991</v>
       </c>
-      <c r="O9" s="106" t="s">
+      <c r="O9" s="105" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="106"/>
-      <c r="Q9" s="106"/>
+      <c r="P9" s="105"/>
+      <c r="Q9" s="105"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
@@ -5721,11 +5771,11 @@
         <f t="shared" ref="M10:M63" si="2">M9-I10</f>
         <v>475943.2699999999</v>
       </c>
-      <c r="O10" s="107" t="s">
+      <c r="O10" s="106" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="107"/>
-      <c r="Q10" s="107"/>
+      <c r="P10" s="106"/>
+      <c r="Q10" s="106"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
@@ -5767,11 +5817,11 @@
         <f t="shared" si="2"/>
         <v>467129.50999999989</v>
       </c>
-      <c r="O11" s="108" t="s">
+      <c r="O11" s="107" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="108"/>
-      <c r="Q11" s="108"/>
+      <c r="P11" s="107"/>
+      <c r="Q11" s="107"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="83" t="s">
@@ -5923,7 +5973,7 @@
         <v>8813.76</v>
       </c>
       <c r="J15" s="77">
-        <f t="shared" ref="J15:J30" si="3">K15-I15</f>
+        <f t="shared" ref="J15:J29" si="3">K15-I15</f>
         <v>906.93000000000029</v>
       </c>
       <c r="K15" s="28">
@@ -6300,12 +6350,10 @@
       <c r="I30" s="28">
         <v>8813.76</v>
       </c>
-      <c r="J30" s="77">
-        <f t="shared" si="3"/>
-        <v>2433.4699999999993</v>
-      </c>
+      <c r="J30" s="77"/>
       <c r="K30" s="28">
-        <v>11247.23</v>
+        <f t="shared" si="1"/>
+        <v>8813.76</v>
       </c>
       <c r="L30" s="29">
         <v>46265</v>
@@ -7087,11 +7135,11 @@
       </c>
       <c r="J64" s="87">
         <f>SUM(J4:J63)</f>
-        <v>31363.22</v>
+        <v>28929.75</v>
       </c>
       <c r="K64" s="87">
         <f>SUM(K4:K63)</f>
-        <v>560189.05000000028</v>
+        <v>557755.58000000019</v>
       </c>
       <c r="L64" s="43"/>
       <c r="M64" s="44"/>
@@ -7486,16 +7534,16 @@
         <v>1110263.04</v>
       </c>
       <c r="P4" s="33">
-        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18+I19+I20+I21+I22+I23+I24</f>
-        <v>388591.98000000004</v>
+        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18+I19+I20+I21+I22+I23</f>
+        <v>370087.60000000003</v>
       </c>
       <c r="Q4" s="34">
         <f>O4-P4</f>
-        <v>721671.06</v>
+        <v>740175.44</v>
       </c>
       <c r="R4" s="34">
         <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29</f>
-        <v>42545.14999999998</v>
+        <v>38411.279999999984</v>
       </c>
     </row>
     <row r="5" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -7579,13 +7627,13 @@
         <f>M5-I6</f>
         <v>1073254.2800000003</v>
       </c>
-      <c r="O6" s="98" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="98"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>Q4/O4-1</f>
-        <v>-0.34999992434225313</v>
+        <v>-0.3333332612783364</v>
       </c>
     </row>
     <row r="7" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -7698,7 +7746,7 @@
         <v>18504.38</v>
       </c>
       <c r="J9" s="28">
-        <f t="shared" ref="J9:J24" si="3">K9-I9</f>
+        <f t="shared" ref="J9:J23" si="3">K9-I9</f>
         <v>928.90999999999985</v>
       </c>
       <c r="K9" s="28">
@@ -7711,11 +7759,11 @@
         <f t="shared" si="2"/>
         <v>1017741.1400000004</v>
       </c>
-      <c r="O9" s="109" t="s">
+      <c r="O9" s="108" t="s">
         <v>86</v>
       </c>
-      <c r="P9" s="109"/>
-      <c r="Q9" s="109"/>
+      <c r="P9" s="108"/>
+      <c r="Q9" s="108"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="79" t="s">
@@ -7757,11 +7805,11 @@
         <f t="shared" si="2"/>
         <v>999236.76000000036</v>
       </c>
-      <c r="O10" s="106" t="s">
+      <c r="O10" s="105" t="s">
         <v>87</v>
       </c>
-      <c r="P10" s="106"/>
-      <c r="Q10" s="106"/>
+      <c r="P10" s="105"/>
+      <c r="Q10" s="105"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="79" t="s">
@@ -7803,11 +7851,11 @@
         <f t="shared" si="2"/>
         <v>980732.38000000035</v>
       </c>
-      <c r="O11" s="107" t="s">
+      <c r="O11" s="106" t="s">
         <v>88</v>
       </c>
-      <c r="P11" s="107"/>
-      <c r="Q11" s="107"/>
+      <c r="P11" s="106"/>
+      <c r="Q11" s="106"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="79" t="s">
@@ -8338,13 +8386,8 @@
       <c r="I24" s="28">
         <v>18504.38</v>
       </c>
-      <c r="J24" s="28">
-        <f t="shared" si="3"/>
-        <v>4133.869999999999</v>
-      </c>
-      <c r="K24" s="28">
-        <v>22638.25</v>
-      </c>
+      <c r="J24" s="28"/>
+      <c r="K24" s="28"/>
       <c r="L24" s="29">
         <v>46265</v>
       </c>
@@ -9677,11 +9720,11 @@
       </c>
       <c r="J64" s="78">
         <f>SUM(J4:J63)</f>
-        <v>42545.14999999998</v>
+        <v>38411.279999999984</v>
       </c>
       <c r="K64" s="78">
         <f>SUM(K4:K63)</f>
-        <v>412632.75</v>
+        <v>389994.5</v>
       </c>
       <c r="L64" s="43"/>
       <c r="M64" s="44"/>
@@ -10601,16 +10644,16 @@
         <v>1786770.79</v>
       </c>
       <c r="P4" s="33">
-        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17+I18</f>
-        <v>446692.65000000008</v>
+        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13+I14+I15+I16+I17</f>
+        <v>416913.14000000007</v>
       </c>
       <c r="Q4" s="34">
         <f>O4-P4</f>
-        <v>1340078.1399999999</v>
+        <v>1369857.65</v>
       </c>
       <c r="R4" s="34">
         <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29</f>
-        <v>36453.030000000021</v>
+        <v>31664.490000000016</v>
       </c>
     </row>
     <row r="5" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -10640,7 +10683,7 @@
         <v>29779.51</v>
       </c>
       <c r="J5" s="77">
-        <f t="shared" ref="J5:J18" si="1">K5-I5</f>
+        <f t="shared" ref="J5:J17" si="1">K5-I5</f>
         <v>297.79000000000087</v>
       </c>
       <c r="K5" s="28">
@@ -10694,13 +10737,13 @@
         <f>M5-I6</f>
         <v>1727211.77</v>
       </c>
-      <c r="O6" s="98" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="98"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
-        <v>-0.24999997341572844</v>
+        <v>-0.23333330852134659</v>
       </c>
     </row>
     <row r="7" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -10828,11 +10871,11 @@
         <f t="shared" ref="M9:M63" si="2">M8-I9</f>
         <v>1637873.24</v>
       </c>
-      <c r="O9" s="106" t="s">
+      <c r="O9" s="105" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="106"/>
-      <c r="Q9" s="106"/>
+      <c r="P9" s="105"/>
+      <c r="Q9" s="105"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="81" t="s">
@@ -10874,11 +10917,11 @@
         <f t="shared" si="2"/>
         <v>1608093.73</v>
       </c>
-      <c r="O10" s="107" t="s">
+      <c r="O10" s="106" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="107"/>
-      <c r="Q10" s="107"/>
+      <c r="P10" s="106"/>
+      <c r="Q10" s="106"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="81" t="s">
@@ -10920,11 +10963,11 @@
         <f t="shared" si="2"/>
         <v>1578314.22</v>
       </c>
-      <c r="O11" s="108" t="s">
+      <c r="O11" s="107" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="108"/>
-      <c r="Q11" s="108"/>
+      <c r="P11" s="107"/>
+      <c r="Q11" s="107"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="81" t="s">
@@ -11169,12 +11212,10 @@
       <c r="I18" s="28">
         <v>29779.51</v>
       </c>
-      <c r="J18" s="77">
-        <f t="shared" si="1"/>
-        <v>4788.5400000000045</v>
-      </c>
+      <c r="J18" s="77"/>
       <c r="K18" s="28">
-        <v>34568.050000000003</v>
+        <f t="shared" ref="K18:K63" si="3">I18+J18</f>
+        <v>29779.51</v>
       </c>
       <c r="L18" s="29">
         <v>45900</v>
@@ -11196,7 +11237,7 @@
       </c>
       <c r="J19" s="77"/>
       <c r="K19" s="28">
-        <f t="shared" ref="K19:K63" si="3">I19+J19</f>
+        <f t="shared" si="3"/>
         <v>29779.51</v>
       </c>
       <c r="L19" s="29">
@@ -12232,11 +12273,11 @@
       </c>
       <c r="J64" s="78">
         <f>SUM(J4:J63)</f>
-        <v>36453.030000000021</v>
+        <v>31664.490000000016</v>
       </c>
       <c r="K64" s="78">
         <f>SUM(K4:K63)</f>
-        <v>1823223.8200000003</v>
+        <v>1818435.2800000003</v>
       </c>
       <c r="L64" s="43"/>
       <c r="M64" s="44"/>
@@ -12634,16 +12675,16 @@
         <v>91297.69</v>
       </c>
       <c r="P4" s="33">
-        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12+I13</f>
-        <v>15216.199999999997</v>
+        <f>I4+I5+I6+I7+I8+I9+I10+I11+I12</f>
+        <v>13694.579999999998</v>
       </c>
       <c r="Q4" s="34">
         <f>O4-P4</f>
-        <v>76081.490000000005</v>
+        <v>77603.11</v>
       </c>
       <c r="R4" s="34">
         <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29</f>
-        <v>744.94000000000096</v>
+        <v>591.41000000000076</v>
       </c>
     </row>
     <row r="5" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -12685,7 +12726,7 @@
         <v>1521.62</v>
       </c>
       <c r="J6" s="77">
-        <f t="shared" ref="J6:J13" si="1">K6-I6</f>
+        <f t="shared" ref="J6:J12" si="1">K6-I6</f>
         <v>33.770000000000209</v>
       </c>
       <c r="K6" s="28">
@@ -12698,13 +12739,13 @@
         <f>M5-I6</f>
         <v>88254.450000000012</v>
       </c>
-      <c r="O6" s="98" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="98"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
-        <v>-0.16666577215699541</v>
+        <v>-0.14999919494129588</v>
       </c>
     </row>
     <row r="7" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -12787,11 +12828,11 @@
         <f t="shared" ref="M9:M63" si="2">M8-I9</f>
         <v>83689.590000000026</v>
       </c>
-      <c r="O9" s="106" t="s">
+      <c r="O9" s="105" t="s">
         <v>87</v>
       </c>
-      <c r="P9" s="106"/>
-      <c r="Q9" s="106"/>
+      <c r="P9" s="105"/>
+      <c r="Q9" s="105"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="39"/>
@@ -12818,11 +12859,11 @@
         <f t="shared" si="2"/>
         <v>82167.97000000003</v>
       </c>
-      <c r="O10" s="107" t="s">
+      <c r="O10" s="106" t="s">
         <v>88</v>
       </c>
-      <c r="P10" s="107"/>
-      <c r="Q10" s="107"/>
+      <c r="P10" s="106"/>
+      <c r="Q10" s="106"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="39"/>
@@ -12849,11 +12890,11 @@
         <f t="shared" si="2"/>
         <v>80646.350000000035</v>
       </c>
-      <c r="O11" s="108" t="s">
+      <c r="O11" s="107" t="s">
         <v>90</v>
       </c>
-      <c r="P11" s="108"/>
-      <c r="Q11" s="108"/>
+      <c r="P11" s="107"/>
+      <c r="Q11" s="107"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="39"/>
@@ -12892,12 +12933,10 @@
       <c r="I13" s="27">
         <v>1521.62</v>
       </c>
-      <c r="J13" s="77">
-        <f t="shared" si="1"/>
-        <v>153.5300000000002</v>
-      </c>
+      <c r="J13" s="77"/>
       <c r="K13" s="28">
-        <v>1675.15</v>
+        <f t="shared" si="0"/>
+        <v>1521.62</v>
       </c>
       <c r="L13" s="29">
         <v>46262</v>
@@ -14454,12 +14493,12 @@
         <v>8285.5799999999963</v>
       </c>
       <c r="P4" s="33">
-        <f>K5+K6</f>
-        <v>516.70000000000005</v>
+        <f>K5+K6+K7+K8+K9+K10+K11+K12+K13+K14+K15</f>
+        <v>2785.48</v>
       </c>
       <c r="Q4" s="34">
         <f>O4-P4</f>
-        <v>7768.8799999999965</v>
+        <v>5500.0999999999967</v>
       </c>
       <c r="R4" s="34">
         <f>J5+J6+J7+J8+J9+J10+J11+J12+J13+J14+J15+J16+J17+J18+J19+J20+J21+J22+J23+J24+J25+J26+J27+J28+J29</f>
@@ -14517,13 +14556,13 @@
         <f>M5-I6</f>
         <v>-501.4</v>
       </c>
-      <c r="O6" s="98" t="s">
+      <c r="O6" s="97" t="s">
         <v>89</v>
       </c>
-      <c r="P6" s="98"/>
+      <c r="P6" s="97"/>
       <c r="Q6" s="82">
         <f>(Q4/O4)-1</f>
-        <v>-6.2361355511623806E-2</v>
+        <v>-0.33618406919008692</v>
       </c>
     </row>
     <row r="7" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
@@ -14603,9 +14642,9 @@
         <f t="shared" ref="M9:M36" si="1">M8-I9</f>
         <v>-1265.98</v>
       </c>
-      <c r="O9" s="99"/>
-      <c r="P9" s="99"/>
-      <c r="Q9" s="99"/>
+      <c r="O9" s="98"/>
+      <c r="P9" s="98"/>
+      <c r="Q9" s="98"/>
     </row>
     <row r="10" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="39"/>
@@ -14630,9 +14669,9 @@
         <f t="shared" si="1"/>
         <v>-1516.68</v>
       </c>
-      <c r="O10" s="99"/>
-      <c r="P10" s="99"/>
-      <c r="Q10" s="99"/>
+      <c r="O10" s="98"/>
+      <c r="P10" s="98"/>
+      <c r="Q10" s="98"/>
     </row>
     <row r="11" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="39"/>
@@ -14657,9 +14696,9 @@
         <f t="shared" si="1"/>
         <v>-1767.38</v>
       </c>
-      <c r="O11" s="99"/>
-      <c r="P11" s="99"/>
-      <c r="Q11" s="99"/>
+      <c r="O11" s="98"/>
+      <c r="P11" s="98"/>
+      <c r="Q11" s="98"/>
     </row>
     <row r="12" spans="2:18" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="39"/>
@@ -15556,30 +15595,30 @@
   <sheetData>
     <row r="1" spans="2:26" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:26" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="111" t="s">
+      <c r="B2" s="110" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="112"/>
-      <c r="D2" s="112"/>
-      <c r="E2" s="112"/>
-      <c r="F2" s="112"/>
-      <c r="G2" s="112"/>
-      <c r="H2" s="112"/>
-      <c r="I2" s="112"/>
-      <c r="J2" s="112"/>
-      <c r="K2" s="112"/>
-      <c r="L2" s="112"/>
-      <c r="M2" s="112"/>
-      <c r="N2" s="112"/>
-      <c r="O2" s="112"/>
-      <c r="P2" s="112"/>
-      <c r="Q2" s="112"/>
-      <c r="R2" s="112"/>
-      <c r="S2" s="112"/>
-      <c r="T2" s="112"/>
-      <c r="U2" s="112"/>
-      <c r="V2" s="112"/>
-      <c r="W2" s="113"/>
+      <c r="C2" s="111"/>
+      <c r="D2" s="111"/>
+      <c r="E2" s="111"/>
+      <c r="F2" s="111"/>
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
+      <c r="J2" s="111"/>
+      <c r="K2" s="111"/>
+      <c r="L2" s="111"/>
+      <c r="M2" s="111"/>
+      <c r="N2" s="111"/>
+      <c r="O2" s="111"/>
+      <c r="P2" s="111"/>
+      <c r="Q2" s="111"/>
+      <c r="R2" s="111"/>
+      <c r="S2" s="111"/>
+      <c r="T2" s="111"/>
+      <c r="U2" s="111"/>
+      <c r="V2" s="111"/>
+      <c r="W2" s="112"/>
     </row>
     <row r="3" spans="2:26" s="4" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="48" t="s">
@@ -16410,8 +16449,8 @@
       <c r="Z22" s="57"/>
     </row>
     <row r="24" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P24" s="110"/>
-      <c r="Q24" s="110"/>
+      <c r="P24" s="109"/>
+      <c r="Q24" s="109"/>
       <c r="R24" s="73"/>
       <c r="S24" s="73"/>
       <c r="T24" s="73"/>
@@ -16420,8 +16459,8 @@
       <c r="W24" s="74"/>
     </row>
     <row r="25" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P25" s="110"/>
-      <c r="Q25" s="110"/>
+      <c r="P25" s="109"/>
+      <c r="Q25" s="109"/>
       <c r="R25" s="73"/>
       <c r="S25" s="73"/>
       <c r="T25" s="73"/>
@@ -16430,8 +16469,8 @@
       <c r="W25" s="74"/>
     </row>
     <row r="26" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P26" s="110"/>
-      <c r="Q26" s="110"/>
+      <c r="P26" s="109"/>
+      <c r="Q26" s="109"/>
       <c r="R26" s="73"/>
       <c r="S26" s="73"/>
       <c r="T26" s="73"/>
@@ -16440,8 +16479,8 @@
       <c r="W26" s="74"/>
     </row>
     <row r="27" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P27" s="110"/>
-      <c r="Q27" s="110"/>
+      <c r="P27" s="109"/>
+      <c r="Q27" s="109"/>
       <c r="R27" s="73"/>
       <c r="S27" s="73"/>
       <c r="T27" s="73"/>
@@ -16450,8 +16489,8 @@
       <c r="W27" s="75"/>
     </row>
     <row r="28" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="P28" s="110"/>
-      <c r="Q28" s="110"/>
+      <c r="P28" s="109"/>
+      <c r="Q28" s="109"/>
       <c r="R28" s="73"/>
       <c r="S28" s="73"/>
       <c r="T28" s="73"/>
@@ -16477,12 +16516,11 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{420301BD-1EC9-404C-9D58-1869DDAA2327}">
-  <dimension ref="B2:P10"/>
+  <dimension ref="B2:P9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="15" width="13.33203125" customWidth="1"/>
-    <col min="16" max="16" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="16" width="13.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.3">
@@ -16525,6 +16563,9 @@
       <c r="O2" s="85">
         <v>46204</v>
       </c>
+      <c r="P2" s="85">
+        <v>46235</v>
+      </c>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B3" s="84" t="s">
@@ -16570,7 +16611,12 @@
       <c r="N3" s="27">
         <v>3912277.58</v>
       </c>
-      <c r="O3" s="27"/>
+      <c r="O3" s="27">
+        <v>5882097.6399999997</v>
+      </c>
+      <c r="P3" s="27">
+        <v>3196894.17</v>
+      </c>
     </row>
     <row r="4" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B4" s="84" t="s">
@@ -16615,6 +16661,9 @@
       <c r="O4" s="27">
         <v>119.3</v>
       </c>
+      <c r="P4" s="27">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B5" s="84" t="s">
@@ -16654,8 +16703,13 @@
       <c r="M5" s="27">
         <v>36214.15</v>
       </c>
-      <c r="N5" s="27"/>
+      <c r="N5" s="27">
+        <v>53315.91</v>
+      </c>
       <c r="O5" s="27"/>
+      <c r="P5" s="27">
+        <v>53315.91</v>
+      </c>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B6" s="84" t="s">
@@ -16683,7 +16737,9 @@
         <f>102854.7</f>
         <v>102854.7</v>
       </c>
-      <c r="J6" s="27"/>
+      <c r="J6" s="27">
+        <v>0</v>
+      </c>
       <c r="K6" s="27">
         <v>0</v>
       </c>
@@ -16691,13 +16747,16 @@
         <v>0</v>
       </c>
       <c r="M6" s="27">
-        <v>166736.70000000001</v>
+        <v>100959.81</v>
       </c>
       <c r="N6" s="27">
         <v>0</v>
       </c>
       <c r="O6" s="27">
         <v>99037.19</v>
+      </c>
+      <c r="P6" s="27">
+        <v>245472</v>
       </c>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.3">
@@ -16733,6 +16792,7 @@
       <c r="M7" s="27"/>
       <c r="N7" s="27"/>
       <c r="O7" s="27"/>
+      <c r="P7" s="27"/>
     </row>
     <row r="8" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B8" s="84" t="s">
@@ -16766,6 +16826,7 @@
       <c r="M8" s="27"/>
       <c r="N8" s="27"/>
       <c r="O8" s="27"/>
+      <c r="P8" s="27"/>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.3">
       <c r="B9" s="84" t="s">
@@ -16813,19 +16874,20 @@
       </c>
       <c r="M9" s="96">
         <f t="shared" si="0"/>
-        <v>202950.85</v>
+        <v>137173.96</v>
       </c>
       <c r="N9" s="96">
         <f t="shared" ref="N9:O9" si="1">SUM(N4:N8)</f>
-        <v>51.02</v>
+        <v>53366.93</v>
       </c>
       <c r="O9" s="96">
         <f t="shared" si="1"/>
         <v>99156.49</v>
       </c>
-    </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.3">
-      <c r="P10" s="97"/>
+      <c r="P9" s="96">
+        <f t="shared" ref="P9" si="2">SUM(P4:P8)</f>
+        <v>298787.91000000003</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>